<commit_message>
feat: expand prototype battle content
</commit_message>
<xml_diff>
--- a/eoe/Assets/Excels/HeroConfig.xlsx
+++ b/eoe/Assets/Excels/HeroConfig.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="16.5" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15.63" customWidth="1" style="2" min="1" max="1"/>
@@ -412,7 +412,7 @@
           <t>critDamage</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="0" t="inlineStr">
         <is>
           <t>lifesteal</t>
         </is>
@@ -469,7 +469,7 @@
       <c r="K2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L2" t="n">
+      <c r="L2" s="0" t="n">
         <v>0</v>
       </c>
       <c r="M2" s="2" t="n">
@@ -479,6 +479,202 @@
         <v>1</v>
       </c>
       <c r="O2" s="2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>102</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>hero.102</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2002</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2002</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2006</v>
+      </c>
+      <c r="F3" t="n">
+        <v>24</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>2</v>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>103</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>hero.103</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2003</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2003</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2007</v>
+      </c>
+      <c r="F4" t="n">
+        <v>18</v>
+      </c>
+      <c r="G4" t="n">
+        <v>7</v>
+      </c>
+      <c r="H4" t="n">
+        <v>4</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>104</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>hero.104</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2004</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2004</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2010</v>
+      </c>
+      <c r="F5" t="n">
+        <v>15</v>
+      </c>
+      <c r="G5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H5" t="n">
+        <v>6</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>2</v>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>105</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>hero.105</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2005</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2005</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2008</v>
+      </c>
+      <c r="F6" t="n">
+        <v>22</v>
+      </c>
+      <c r="G6" t="n">
+        <v>6</v>
+      </c>
+      <c r="H6" t="n">
+        <v>3</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>2</v>
+      </c>
+      <c r="N6" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
         <v>5</v>
       </c>
     </row>

</xml_diff>